<commit_message>
update sensitivity analysis experiment
</commit_message>
<xml_diff>
--- a/Sensitivity analysis/figure6.xlsx
+++ b/Sensitivity analysis/figure6.xlsx
@@ -425,37 +425,37 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.2065986394557823</v>
+        <v>0.07675</v>
       </c>
       <c r="C2">
-        <v>0.2068934240362812</v>
+        <v>0.07675</v>
       </c>
       <c r="D2">
-        <v>0.2073696145124717</v>
+        <v>0.076475</v>
       </c>
       <c r="E2">
-        <v>0.2086621315192744</v>
+        <v>0.076225</v>
       </c>
       <c r="F2">
-        <v>0.2099092970521542</v>
+        <v>0.076275</v>
       </c>
       <c r="G2">
-        <v>0.2110430839002267</v>
+        <v>0.07655000000000001</v>
       </c>
       <c r="H2">
-        <v>0.2118367346938775</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="I2">
-        <v>0.2133106575963719</v>
+        <v>0.07704999999999999</v>
       </c>
       <c r="J2">
-        <v>0.2143310657596372</v>
+        <v>0.0772</v>
       </c>
       <c r="K2">
-        <v>0.2151473922902494</v>
+        <v>0.07785</v>
       </c>
       <c r="L2">
-        <v>0.2166213151927438</v>
+        <v>0.07875</v>
       </c>
     </row>
     <row r="3">
@@ -465,37 +465,37 @@
         </is>
       </c>
       <c r="B3">
-        <v>0.8355328798185941</v>
+        <v>0.267125</v>
       </c>
       <c r="C3">
-        <v>0.8364172335600907</v>
+        <v>0.262025</v>
       </c>
       <c r="D3">
-        <v>0.8375283446712019</v>
+        <v>0.2513</v>
       </c>
       <c r="E3">
-        <v>0.8393877551020408</v>
+        <v>0.235275</v>
       </c>
       <c r="F3">
-        <v>0.8411111111111111</v>
+        <v>0.217075</v>
       </c>
       <c r="G3">
-        <v>0.8423129251700681</v>
+        <v>0.199125</v>
       </c>
       <c r="H3">
-        <v>0.8441043083900227</v>
+        <v>0.18005</v>
       </c>
       <c r="I3">
-        <v>0.8454421768707483</v>
+        <v>0.163925</v>
       </c>
       <c r="J3">
-        <v>0.8466893424036281</v>
+        <v>0.14715</v>
       </c>
       <c r="K3">
-        <v>0.8480045351473923</v>
+        <v>0.1332</v>
       </c>
       <c r="L3">
-        <v>0.849092970521542</v>
+        <v>0.121825</v>
       </c>
     </row>
   </sheetData>
@@ -577,37 +577,37 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.2065986394557823</v>
+        <v>0.07675</v>
       </c>
       <c r="C2">
-        <v>0.1617913832199546</v>
+        <v>0.07665</v>
       </c>
       <c r="D2">
-        <v>0.1631065759637188</v>
+        <v>0.07615</v>
       </c>
       <c r="E2">
-        <v>0.1773922902494331</v>
+        <v>0.07502499999999999</v>
       </c>
       <c r="F2">
-        <v>0.2002947845804989</v>
+        <v>0.0738</v>
       </c>
       <c r="G2">
-        <v>0.2337414965986395</v>
+        <v>0.0746</v>
       </c>
       <c r="H2">
-        <v>0.2700226757369614</v>
+        <v>0.075625</v>
       </c>
       <c r="I2">
-        <v>0.3033560090702948</v>
+        <v>0.07665</v>
       </c>
       <c r="J2">
-        <v>0.3261224489795919</v>
+        <v>0.075725</v>
       </c>
       <c r="K2">
-        <v>0.2247392290249433</v>
+        <v>0.049025</v>
       </c>
       <c r="L2">
-        <v>0.3666439909297052</v>
+        <v>0.07845000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -617,37 +617,37 @@
         </is>
       </c>
       <c r="B3">
-        <v>0.8355328798185941</v>
+        <v>0.267125</v>
       </c>
       <c r="C3">
-        <v>0.8350340136054422</v>
+        <v>0.268025</v>
       </c>
       <c r="D3">
-        <v>0.834920634920635</v>
+        <v>0.2692</v>
       </c>
       <c r="E3">
-        <v>0.8345804988662131</v>
+        <v>0.27035</v>
       </c>
       <c r="F3">
-        <v>0.83437641723356</v>
+        <v>0.271525</v>
       </c>
       <c r="G3">
-        <v>0.8342857142857143</v>
+        <v>0.272775</v>
       </c>
       <c r="H3">
-        <v>0.8341269841269842</v>
+        <v>0.2739</v>
       </c>
       <c r="I3">
-        <v>0.8342176870748299</v>
+        <v>0.274925</v>
       </c>
       <c r="J3">
-        <v>0.8343990929705215</v>
+        <v>0.2766</v>
       </c>
       <c r="K3">
-        <v>0.8348526077097506</v>
+        <v>0.279475</v>
       </c>
       <c r="L3">
-        <v>0.8353061224489796</v>
+        <v>0.2815</v>
       </c>
     </row>
   </sheetData>
@@ -729,37 +729,37 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.2065986394557823</v>
+        <v>0.07675</v>
       </c>
       <c r="C2">
-        <v>0.1619274376417233</v>
+        <v>0.0767</v>
       </c>
       <c r="D2">
-        <v>0.1636507936507937</v>
+        <v>0.076275</v>
       </c>
       <c r="E2">
-        <v>0.1780498866213152</v>
+        <v>0.07552499999999999</v>
       </c>
       <c r="F2">
-        <v>0.2014965986394558</v>
+        <v>0.07527499999999999</v>
       </c>
       <c r="G2">
-        <v>0.2358503401360544</v>
+        <v>0.077125</v>
       </c>
       <c r="H2">
-        <v>0.2743310657596372</v>
+        <v>0.079275</v>
       </c>
       <c r="I2">
-        <v>0.3097505668934241</v>
+        <v>0.0815</v>
       </c>
       <c r="J2">
-        <v>0.3349886621315193</v>
+        <v>0.08155</v>
       </c>
       <c r="K2">
-        <v>0.2343764172335601</v>
+        <v>0.05205</v>
       </c>
       <c r="L2">
-        <v>0.3809297052154195</v>
+        <v>0.08497499999999999</v>
       </c>
     </row>
     <row r="3">
@@ -769,37 +769,37 @@
         </is>
       </c>
       <c r="B3">
-        <v>0.8355328798185941</v>
+        <v>0.267125</v>
       </c>
       <c r="C3">
-        <v>0.8360090702947846</v>
+        <v>0.26315</v>
       </c>
       <c r="D3">
-        <v>0.8368934240362812</v>
+        <v>0.253775</v>
       </c>
       <c r="E3">
-        <v>0.8384126984126984</v>
+        <v>0.23895</v>
       </c>
       <c r="F3">
-        <v>0.8400226757369614</v>
+        <v>0.221925</v>
       </c>
       <c r="G3">
-        <v>0.8415646258503401</v>
+        <v>0.20505</v>
       </c>
       <c r="H3">
-        <v>0.8441043083900227</v>
+        <v>0.18755</v>
       </c>
       <c r="I3">
-        <v>0.8456235827664399</v>
+        <v>0.171925</v>
       </c>
       <c r="J3">
-        <v>0.846530612244898</v>
+        <v>0.156225</v>
       </c>
       <c r="K3">
-        <v>0.8479591836734693</v>
+        <v>0.144025</v>
       </c>
       <c r="L3">
-        <v>0.8497959183673469</v>
+        <v>0.13415</v>
       </c>
     </row>
   </sheetData>

</xml_diff>